<commit_message>
Add full page suite, expanded backend API, and grading module
- Added 10 new pages: Dashboard, Categories, DividendAnalysis, DividendCalendar,
  ETFScreen, Growth, NavErosion, NavErosionPortfolio, PortfolioIncomeSim,
  BuySellSignals, TotalReturn, Settings, Watchlist
- Major expansion of Flask API (app.py) with endpoints for all new pages
- Added backend/grading.py for portfolio grading logic
- Updated App.jsx routing and nav to include all new pages
- Expanded index.css with full app styling
- Updated import, holdings, database, and template files
- Added .claude/ to .gitignore to exclude local AI memory

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/portfolio_upload_template.xlsx
+++ b/templates/portfolio_upload_template.xlsx
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF4"/>
+  <dimension ref="A1:AH4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -469,21 +469,23 @@
     <col width="15" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="19" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="19" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
     <col width="17" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="23" customWidth="1" min="24" max="24"/>
-    <col width="19" customWidth="1" min="25" max="25"/>
-    <col width="21" customWidth="1" min="26" max="26"/>
-    <col width="19" customWidth="1" min="27" max="27"/>
+    <col width="17" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="23" customWidth="1" min="25" max="25"/>
+    <col width="19" customWidth="1" min="26" max="26"/>
+    <col width="21" customWidth="1" min="27" max="27"/>
     <col width="19" customWidth="1" min="28" max="28"/>
-    <col width="15" customWidth="1" min="29" max="29"/>
-    <col width="16" customWidth="1" min="30" max="30"/>
-    <col width="19" customWidth="1" min="31" max="31"/>
-    <col width="20" customWidth="1" min="32" max="32"/>
+    <col width="19" customWidth="1" min="29" max="29"/>
+    <col width="15" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="19" customWidth="1" min="32" max="32"/>
+    <col width="20" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,87 +566,97 @@
       </c>
       <c r="P1" s="2" t="inlineStr">
         <is>
+          <t>Pay Date</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
           <t>DRIP</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>Div Paid</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>Est. Annual Pmt</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>Monthly Income</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>Yield On Cost</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>Current Yield</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>% of Account</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>YTD Divs</t>
         </is>
       </c>
-      <c r="X1" s="2" t="inlineStr">
+      <c r="Y1" s="2" t="inlineStr">
         <is>
           <t>Total Divs Received</t>
         </is>
       </c>
-      <c r="Y1" s="2" t="inlineStr">
+      <c r="Z1" s="2" t="inlineStr">
         <is>
           <t>Paid For Itself</t>
         </is>
       </c>
-      <c r="Z1" s="2" t="inlineStr">
+      <c r="AA1" s="2" t="inlineStr">
         <is>
           <t>Cash Not Reinvest</t>
         </is>
       </c>
-      <c r="AA1" s="2" t="inlineStr">
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>Cash Reinvested</t>
         </is>
       </c>
-      <c r="AB1" s="2" t="inlineStr">
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>Shares from Div</t>
         </is>
       </c>
-      <c r="AC1" s="2" t="inlineStr">
+      <c r="AD1" s="2" t="inlineStr">
         <is>
           <t>Shares/Year</t>
         </is>
       </c>
-      <c r="AD1" s="2" t="inlineStr">
+      <c r="AE1" s="2" t="inlineStr">
         <is>
           <t>Shares/Month</t>
         </is>
       </c>
-      <c r="AE1" s="2" t="inlineStr">
+      <c r="AF1" s="2" t="inlineStr">
         <is>
           <t>8% Annual Wdraw</t>
         </is>
       </c>
-      <c r="AF1" s="2" t="inlineStr">
+      <c r="AG1" s="2" t="inlineStr">
         <is>
           <t>8% Monthly Wdraw</t>
+        </is>
+      </c>
+      <c r="AH1" s="2" t="inlineStr">
+        <is>
+          <t>Category</t>
         </is>
       </c>
     </row>
@@ -691,16 +703,21 @@
           <t>03/01/25</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="W2" s="3" t="n">
+      <c r="X2" s="3" t="n">
         <v>135</v>
       </c>
-      <c r="X2" s="3" t="n">
+      <c r="Y2" s="3" t="n">
         <v>540</v>
+      </c>
+      <c r="AH2" s="3" t="inlineStr">
+        <is>
+          <t>Anchors</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -746,16 +763,21 @@
           <t>03/15/25</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="W3" s="3" t="n">
+      <c r="X3" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="X3" s="3" t="n">
+      <c r="Y3" s="3" t="n">
         <v>186</v>
+      </c>
+      <c r="AH3" s="3" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -801,16 +823,21 @@
           <t>02/28/25</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="W4" s="3" t="n">
+      <c r="X4" s="3" t="n">
         <v>19.5</v>
       </c>
-      <c r="X4" s="3" t="n">
+      <c r="Y4" s="3" t="n">
         <v>78</v>
+      </c>
+      <c r="AH4" s="3" t="inlineStr">
+        <is>
+          <t>Boosters</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -824,7 +851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1107,7 +1134,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DRIP</t>
+          <t>Pay Date</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1117,14 +1144,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dividend reinvestment: Y=Yes, N=No (defaults to N)</t>
+          <t>Dividend payment date (auto-estimated as ex-div + 3 weeks if blank)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Div Paid</t>
+          <t>DRIP</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1134,14 +1161,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Total dividends paid to date</t>
+          <t>Dividend reinvestment: Y=Yes, N=No (defaults to N)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Est. Annual Pmt</t>
+          <t>Div Paid</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1151,14 +1178,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Estimated annual dividend payment (auto-calculated as Div/Share x Shares if blank)</t>
+          <t>Total dividends paid to date</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Monthly Income</t>
+          <t>Est. Annual Pmt</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1168,14 +1195,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Approximate monthly dividend income (auto-calculated if blank)</t>
+          <t>Estimated annual dividend payment (auto-calculated as Div/Share x Shares if blank)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Yield On Cost</t>
+          <t>Monthly Income</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1185,14 +1212,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Annual yield based on price paid (auto-calculated if blank)</t>
+          <t>Approximate monthly dividend income (auto-calculated if blank)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Current Yield</t>
+          <t>Yield On Cost</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1202,14 +1229,14 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Annual yield based on current price (auto-calculated if blank)</t>
+          <t>Annual yield based on price paid (auto-calculated if blank)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>% of Account</t>
+          <t>Current Yield</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1219,14 +1246,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Position weight as percentage of total portfolio</t>
+          <t>Annual yield based on current price (auto-calculated if blank)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>YTD Divs</t>
+          <t>% of Account</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1236,14 +1263,14 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Year-to-date dividends received</t>
+          <t>Position weight as percentage of total portfolio</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Total Divs Received</t>
+          <t>YTD Divs</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1253,14 +1280,14 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Total lifetime dividends received from this position</t>
+          <t>Year-to-date dividends received</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Paid For Itself</t>
+          <t>Total Divs Received</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1270,14 +1297,14 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ratio of total dividends received to purchase value</t>
+          <t>Total lifetime dividends received from this position</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Cash Not Reinvest</t>
+          <t>Paid For Itself</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1287,14 +1314,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Cash dividends not reinvested</t>
+          <t>Ratio of total dividends received to purchase value</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Cash Reinvested</t>
+          <t>Cash Not Reinvest</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1304,14 +1331,14 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Total cash dividends that were reinvested</t>
+          <t>Cash dividends not reinvested</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Shares from Div</t>
+          <t>Cash Reinvested</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1321,14 +1348,14 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Number of shares acquired through DRIP</t>
+          <t>Total cash dividends that were reinvested</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Shares/Year</t>
+          <t>Shares from Div</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1338,14 +1365,14 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Shares bought per year from dividends</t>
+          <t>Number of shares acquired through DRIP</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Shares/Month</t>
+          <t>Shares/Year</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1355,14 +1382,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Shares bought per month from dividends</t>
+          <t>Shares bought per year from dividends</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>8% Annual Wdraw</t>
+          <t>Shares/Month</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1372,24 +1399,58 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Annual withdrawal amount at 8% rate</t>
+          <t>Shares bought per month from dividends</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>8% Annual Wdraw</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Annual withdrawal amount at 8% rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>8% Monthly Wdraw</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>Monthly withdrawal amount at 8% rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Category name to assign this ticker to (e.g., Anchors, Boosters, Growth). Creates category if it doesn't exist.</t>
         </is>
       </c>
     </row>

</xml_diff>